<commit_message>
balck and white version
</commit_message>
<xml_diff>
--- a/parties_topics.xlsx
+++ b/parties_topics.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="59">
   <si>
     <t>Country</t>
   </si>
@@ -155,9 +155,6 @@
   </si>
   <si>
     <t>DP</t>
-  </si>
-  <si>
-    <t>euroskpticism</t>
   </si>
   <si>
     <t>https://danskfolkeparti.dk/vores-politik/</t>
@@ -966,22 +963,22 @@
         <v>14</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>35</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M9" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>50</v>
       </c>
       <c r="C10" s="6">
         <v>35</v>
@@ -1008,19 +1005,19 @@
         <v>35</v>
       </c>
       <c r="K10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="L10" s="8" t="s">
         <v>51</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="M10" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="32.25">
       <c r="A11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>54</v>
       </c>
       <c r="C11" s="6">
         <v>54</v>
@@ -1047,19 +1044,19 @@
         <v>31</v>
       </c>
       <c r="K11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L11" s="8" t="s">
         <v>55</v>
-      </c>
-      <c r="L11" s="8" t="s">
-        <v>56</v>
       </c>
       <c r="M11" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="C12" s="6">
         <v>14</v>
@@ -1089,7 +1086,7 @@
         <v>26</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M12" s="5"/>
     </row>

</xml_diff>